<commit_message>
Kashmir v3.4.4 assurance: 2 blind-audit coordinate fixes + refreshed assets
Independent blind re-verification surfaced two endpoint-coordinate errors that
were re-geocoded and re-routed (Batamaloo->Manigam 54.5->37.1 km, SSCL fleet 13
kept; Hazratbal/Lalbazar origin to the real shrine). Refreshed routes/impact/log
JSON + CSV/GeoJSON + all v3.4.4 workbooks from the corrected plan. Fleet total
unchanged at 1,004 (186 active).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.4.4_RTO.xlsx
+++ b/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.4.4_RTO.xlsx
@@ -918,7 +918,7 @@
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Version: v3.4.3  |  Generated: 25 Jun 2026</t>
+          <t>Version: v3.4.3  |  Generated: 26 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -24943,10 +24943,10 @@
         </is>
       </c>
       <c r="G216" s="49" t="n">
-        <v>6.5</v>
+        <v>6.356</v>
       </c>
       <c r="H216" s="47" t="n">
-        <v>52</v>
+        <v>50.8</v>
       </c>
       <c r="I216" s="47" t="n">
         <v>35</v>
@@ -71275,10 +71275,10 @@
         </is>
       </c>
       <c r="G642" s="69" t="n">
-        <v>54.466</v>
+        <v>37.093</v>
       </c>
       <c r="H642" s="67" t="n">
-        <v>163.4</v>
+        <v>111.3</v>
       </c>
       <c r="I642" s="67" t="n">
         <v>15</v>
@@ -84789,7 +84789,7 @@
       </c>
       <c r="C5" s="85" t="inlineStr">
         <is>
-          <t>25 Jun 2026</t>
+          <t>26 Jun 2026</t>
         </is>
       </c>
     </row>

</xml_diff>